<commit_message>
Add remaining vendors to Scrap Vendors sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XVi8LRrXHdPJmY1JXLxuUU
</commit_message>
<xml_diff>
--- a/Private_Scrap_Auction_Links_updated.xlsx
+++ b/Private_Scrap_Auction_Links_updated.xlsx
@@ -14,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Highly Relevant'!$A$4:$L$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Less Relevant'!$A$4:$L$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scrap Vendors'!$A$4:$G$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scrap Vendors'!$A$4:$G$42</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -5079,7 +5079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="15" min="1" max="1"/>
@@ -5918,8 +5918,568 @@
         </is>
       </c>
     </row>
+    <row r="27" ht="44" customHeight="1" s="15">
+      <c r="A27" s="23" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>Metcast India</t>
+        </is>
+      </c>
+      <c r="C27" s="25" t="inlineStr">
+        <is>
+          <t>Howrah, West Bengal</t>
+        </is>
+      </c>
+      <c r="D27" s="25" t="inlineStr">
+        <is>
+          <t>Bronze, brass and gunmetal scrap (listed at Rs 900/kg, 100 kg minimum; price not verified)</t>
+        </is>
+      </c>
+      <c r="E27" s="26" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/impcat/bronze-scrap.html</t>
+        </is>
+      </c>
+      <c r="F27" s="25" t="inlineStr">
+        <is>
+          <t>IndiaMART category page (no direct profile link found)</t>
+        </is>
+      </c>
+      <c r="G27" s="25" t="inlineStr">
+        <is>
+          <t>Open the category page and search the name</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="44" customHeight="1" s="15">
+      <c r="A28" s="27" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>Ronak Enterprise</t>
+        </is>
+      </c>
+      <c r="C28" s="29" t="inlineStr">
+        <is>
+          <t>Bhavnagar, Gujarat</t>
+        </is>
+      </c>
+      <c r="D28" s="29" t="inlineStr">
+        <is>
+          <t>Gunmetal bronze scrap (listed at Rs 900/kg in 50 kg packs; price not verified)</t>
+        </is>
+      </c>
+      <c r="E28" s="30" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/impcat/bronze-scrap.html</t>
+        </is>
+      </c>
+      <c r="F28" s="29" t="inlineStr">
+        <is>
+          <t>IndiaMART category page (no direct profile link found)</t>
+        </is>
+      </c>
+      <c r="G28" s="29" t="inlineStr">
+        <is>
+          <t>Open the category page and search the name</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="44" customHeight="1" s="15">
+      <c r="A29" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>Gaurav Steel</t>
+        </is>
+      </c>
+      <c r="C29" s="25" t="inlineStr">
+        <is>
+          <t>Kolkata, West Bengal</t>
+        </is>
+      </c>
+      <c r="D29" s="25" t="inlineStr">
+        <is>
+          <t>Phosphor bronze scrap (listed at Rs 750/kg in 50 kg bags; price not verified)</t>
+        </is>
+      </c>
+      <c r="E29" s="26" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/impcat/bronze-scrap.html</t>
+        </is>
+      </c>
+      <c r="F29" s="25" t="inlineStr">
+        <is>
+          <t>IndiaMART category page (no direct profile link found)</t>
+        </is>
+      </c>
+      <c r="G29" s="25" t="inlineStr">
+        <is>
+          <t>Open the category page and search the name</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="44" customHeight="1" s="15">
+      <c r="A30" s="27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="28" t="inlineStr">
+        <is>
+          <t>Prashaant Steel &amp; Alloys</t>
+        </is>
+      </c>
+      <c r="C30" s="29" t="inlineStr">
+        <is>
+          <t>Madhavbaug, Mumbai</t>
+        </is>
+      </c>
+      <c r="D30" s="29" t="inlineStr">
+        <is>
+          <t>Phosphor bronze blocks and ingots (listed at Rs 600/kg); ingot, not scrap</t>
+        </is>
+      </c>
+      <c r="E30" s="30" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/impcat/bronze-ingots.html</t>
+        </is>
+      </c>
+      <c r="F30" s="29" t="inlineStr">
+        <is>
+          <t>IndiaMART category page</t>
+        </is>
+      </c>
+      <c r="G30" s="29" t="inlineStr">
+        <is>
+          <t>Ingot source, useful as a price comparison with scrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="44" customHeight="1" s="15">
+      <c r="A31" s="23" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>Supreme Metals</t>
+        </is>
+      </c>
+      <c r="C31" s="25" t="inlineStr">
+        <is>
+          <t>India (location not confirmed)</t>
+        </is>
+      </c>
+      <c r="D31" s="25" t="inlineStr">
+        <is>
+          <t>Metal trader appearing in brass and bronze scrap searches</t>
+        </is>
+      </c>
+      <c r="E31" s="26" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/supreme-metals/testimonial.html</t>
+        </is>
+      </c>
+      <c r="F31" s="25" t="inlineStr">
+        <is>
+          <t>IndiaMART listing</t>
+        </is>
+      </c>
+      <c r="G31" s="25" t="inlineStr">
+        <is>
+          <t>Confirm location and which scrap grades are stocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="44" customHeight="1" s="15">
+      <c r="A32" s="27" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>Laxmi Alloys Casting Co</t>
+        </is>
+      </c>
+      <c r="C32" s="29" t="inlineStr">
+        <is>
+          <t>India (location not confirmed)</t>
+        </is>
+      </c>
+      <c r="D32" s="29" t="inlineStr">
+        <is>
+          <t>Alloy casting company appearing in gunmetal and bronze searches</t>
+        </is>
+      </c>
+      <c r="E32" s="30" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/laxmi-alloys-casting-co-9667818/</t>
+        </is>
+      </c>
+      <c r="F32" s="29" t="inlineStr">
+        <is>
+          <t>TradeIndia listing</t>
+        </is>
+      </c>
+      <c r="G32" s="29" t="inlineStr">
+        <is>
+          <t>Foundry; confirm whether it sells scrap or only castings</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="44" customHeight="1" s="15">
+      <c r="A33" s="23" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>Kqer Manglam Metals</t>
+        </is>
+      </c>
+      <c r="C33" s="25" t="inlineStr">
+        <is>
+          <t>India (location not confirmed)</t>
+        </is>
+      </c>
+      <c r="D33" s="25" t="inlineStr">
+        <is>
+          <t>Copper alloy supplier appearing in bronze scrap searches</t>
+        </is>
+      </c>
+      <c r="E33" s="26" t="inlineStr">
+        <is>
+          <t>https://matmatch.com/suppliers/kqer-manglam-metals</t>
+        </is>
+      </c>
+      <c r="F33" s="25" t="inlineStr">
+        <is>
+          <t>Matmatch profile</t>
+        </is>
+      </c>
+      <c r="G33" s="25" t="inlineStr">
+        <is>
+          <t>Confirm products and location</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="44" customHeight="1" s="15">
+      <c r="A34" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>Enlighten Businesses Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="inlineStr">
+        <is>
+          <t>Dared, Jamnagar, Gujarat</t>
+        </is>
+      </c>
+      <c r="D34" s="29" t="inlineStr">
+        <is>
+          <t>Gunmetal scrap</t>
+        </is>
+      </c>
+      <c r="E34" s="30" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/indian-suppliers/gunmetal-scrap.htm</t>
+        </is>
+      </c>
+      <c r="F34" s="29" t="inlineStr">
+        <is>
+          <t>ExportersIndia listing</t>
+        </is>
+      </c>
+      <c r="G34" s="29" t="inlineStr">
+        <is>
+          <t>Confirm grades and minimum quantity</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="44" customHeight="1" s="15">
+      <c r="A35" s="23" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>Kernel Serviced</t>
+        </is>
+      </c>
+      <c r="C35" s="25" t="inlineStr">
+        <is>
+          <t>Noida, Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="D35" s="25" t="inlineStr">
+        <is>
+          <t>Gunmetal scrap for foundry use (no price shown)</t>
+        </is>
+      </c>
+      <c r="E35" s="26" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/indian-suppliers/gunmetal-scrap.htm</t>
+        </is>
+      </c>
+      <c r="F35" s="25" t="inlineStr">
+        <is>
+          <t>ExportersIndia listing</t>
+        </is>
+      </c>
+      <c r="G35" s="25" t="inlineStr">
+        <is>
+          <t>Delhi NCR; confirm grade and price</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="44" customHeight="1" s="15">
+      <c r="A36" s="27" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="28" t="inlineStr">
+        <is>
+          <t>Rajesh Metal Syndicate</t>
+        </is>
+      </c>
+      <c r="C36" s="29" t="inlineStr">
+        <is>
+          <t>Mumbai, Maharashtra</t>
+        </is>
+      </c>
+      <c r="D36" s="29" t="inlineStr">
+        <is>
+          <t>Commercial gunmetal scrap (listed at Rs 41/kg, 100 kg minimum; price looks unusually low, verify)</t>
+        </is>
+      </c>
+      <c r="E36" s="30" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/indian-suppliers/gunmetal-scrap.htm</t>
+        </is>
+      </c>
+      <c r="F36" s="29" t="inlineStr">
+        <is>
+          <t>ExportersIndia listing</t>
+        </is>
+      </c>
+      <c r="G36" s="29" t="inlineStr">
+        <is>
+          <t>Verify price and metal content</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="44" customHeight="1" s="15">
+      <c r="A37" s="23" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="24" t="inlineStr">
+        <is>
+          <t>Shanky Group</t>
+        </is>
+      </c>
+      <c r="C37" s="25" t="inlineStr">
+        <is>
+          <t>Ashok Vihar, Delhi</t>
+        </is>
+      </c>
+      <c r="D37" s="25" t="inlineStr">
+        <is>
+          <t>Brass scrap</t>
+        </is>
+      </c>
+      <c r="E37" s="26" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/delhi/brass-scrap.htm</t>
+        </is>
+      </c>
+      <c r="F37" s="25" t="inlineStr">
+        <is>
+          <t>ExportersIndia listing</t>
+        </is>
+      </c>
+      <c r="G37" s="25" t="inlineStr">
+        <is>
+          <t>Delhi NCR; ask for sample assay</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="44" customHeight="1" s="15">
+      <c r="A38" s="27" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="28" t="inlineStr">
+        <is>
+          <t>Vansi Iron Traders</t>
+        </is>
+      </c>
+      <c r="C38" s="29" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D38" s="29" t="inlineStr">
+        <is>
+          <t>Scrap trader appearing in the Delhi brass scrap listing</t>
+        </is>
+      </c>
+      <c r="E38" s="30" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/delhi/brass-scrap.htm</t>
+        </is>
+      </c>
+      <c r="F38" s="29" t="inlineStr">
+        <is>
+          <t>ExportersIndia listing</t>
+        </is>
+      </c>
+      <c r="G38" s="29" t="inlineStr">
+        <is>
+          <t>Confirm non-ferrous grades stocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="44" customHeight="1" s="15">
+      <c r="A39" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>Prism Metals</t>
+        </is>
+      </c>
+      <c r="C39" s="25" t="inlineStr">
+        <is>
+          <t>B-28 Mayapuri Industrial Area, Phase-1, New Delhi</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="inlineStr">
+        <is>
+          <t>Brass products manufacturer (not a scrap dealer)</t>
+        </is>
+      </c>
+      <c r="E39" s="26" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/delhi/brass-scrap.htm</t>
+        </is>
+      </c>
+      <c r="F39" s="25" t="inlineStr">
+        <is>
+          <t>ExportersIndia listing</t>
+        </is>
+      </c>
+      <c r="G39" s="25" t="inlineStr">
+        <is>
+          <t>Possible buyer or source of brass offcuts; confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="44" customHeight="1" s="15">
+      <c r="A40" s="27" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="28" t="inlineStr">
+        <is>
+          <t>S.D. Industrial Corporation</t>
+        </is>
+      </c>
+      <c r="C40" s="29" t="inlineStr">
+        <is>
+          <t>India (location not confirmed)</t>
+        </is>
+      </c>
+      <c r="D40" s="29" t="inlineStr">
+        <is>
+          <t>Aluminium alloy wheel, 6063, wire and UBC scrap</t>
+        </is>
+      </c>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>https://www.alcircle.com/biz/verified-aluminium-suppliers?pageNo=8</t>
+        </is>
+      </c>
+      <c r="F40" s="29" t="inlineStr">
+        <is>
+          <t>alCircle verified-supplier list</t>
+        </is>
+      </c>
+      <c r="G40" s="29" t="inlineStr">
+        <is>
+          <t>Aluminium source for aluminium bronze; confirm grades</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="44" customHeight="1" s="15">
+      <c r="A41" s="23" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="24" t="inlineStr">
+        <is>
+          <t>Elevare Exports and Imports</t>
+        </is>
+      </c>
+      <c r="C41" s="25" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="D41" s="25" t="inlineStr">
+        <is>
+          <t>Aluminium extrusion scrap 6063/6061 (1 MT minimum)</t>
+        </is>
+      </c>
+      <c r="E41" s="26" t="inlineStr">
+        <is>
+          <t>https://www.globallinker.com/seller/elevare-exports-and-imports</t>
+        </is>
+      </c>
+      <c r="F41" s="25" t="inlineStr">
+        <is>
+          <t>GlobalLinker profile</t>
+        </is>
+      </c>
+      <c r="G41" s="25" t="inlineStr">
+        <is>
+          <t>New company (established 2025) and IEC code not shown, so verify before ordering</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="44" customHeight="1" s="15">
+      <c r="A42" s="27" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="28" t="inlineStr">
+        <is>
+          <t>Century Metal Recycling Ltd</t>
+        </is>
+      </c>
+      <c r="C42" s="29" t="inlineStr">
+        <is>
+          <t>Faridabad, Haryana</t>
+        </is>
+      </c>
+      <c r="D42" s="29" t="inlineStr">
+        <is>
+          <t>Aluminium and zinc alloy recycler; sells ingot or molten metal (no copper or brass)</t>
+        </is>
+      </c>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>https://www.instafinancials.com/company/century-metal-recycling-limited/U74899HR1994PLC086105</t>
+        </is>
+      </c>
+      <c r="F42" s="29" t="inlineStr">
+        <is>
+          <t>Company registry page (own website not found)</t>
+        </is>
+      </c>
+      <c r="G42" s="29" t="inlineStr">
+        <is>
+          <t>Aluminium alloy source only; check current legal status</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G26"/>
+  <autoFilter ref="A4:G42"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
@@ -5946,6 +6506,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Vendor List sheet with all 38 vendors
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XVi8LRrXHdPJmY1JXLxuUU
</commit_message>
<xml_diff>
--- a/Private_Scrap_Auction_Links_updated.xlsx
+++ b/Private_Scrap_Auction_Links_updated.xlsx
@@ -9,12 +9,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Highly Relevant" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Less Relevant" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scrap Vendors" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendor List" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Highly Relevant'!$A$4:$L$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Less Relevant'!$A$4:$L$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scrap Vendors'!$A$4:$G$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Vendor List'!$A$4:$E$42</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -6530,6 +6532,1067 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E7D32"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" style="15" min="1" max="1"/>
+    <col width="32" customWidth="1" style="15" min="2" max="2"/>
+    <col width="30" customWidth="1" style="15" min="3" max="3"/>
+    <col width="50" customWidth="1" style="15" min="4" max="4"/>
+    <col width="60" customWidth="1" style="15" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Vendor list: all 38 scrap vendors (name and website link)</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="n"/>
+      <c r="C1" s="20" t="n"/>
+      <c r="D1" s="20" t="n"/>
+      <c r="E1" s="20" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" s="15">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>Scrap covered: copper, brass, bronze, gunmetal and aluminium (for aluminium bronze). Details and checks for each vendor are on the Scrap Vendors sheet. Contact details and prices are not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1" s="15">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>Vendor name</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>City / state</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>Scrap they offer</t>
+        </is>
+      </c>
+      <c r="E4" s="22" t="inlineStr">
+        <is>
+          <t>Website link</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1" s="15">
+      <c r="A5" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Gravita India Ltd</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>Mundra and other plants, Gujarat</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="inlineStr">
+        <is>
+          <t>Copper and copper-alloy scrap recycler; also processes lead and aluminium</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>https://www.gravitaindia.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1" s="15">
+      <c r="A6" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>Pramukh Import Export</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>India (customs clearance at Mundra, JNPT, Chennai)</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
+        <is>
+          <t>Aluminium, copper and brass scrap, imported</t>
+        </is>
+      </c>
+      <c r="E6" s="30" t="inlineStr">
+        <is>
+          <t>https://pramukhimportexport.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1" s="15">
+      <c r="A7" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Aryan Recycling</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>Gujarat (processing yard)</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>Scrap metal importer and recycler: aluminium, copper, brass</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>https://www.aryanrecycling.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1" s="15">
+      <c r="A8" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>Jain Metal Group</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
+        <is>
+          <t>Copper scrap and other metals; scrap import trading</t>
+        </is>
+      </c>
+      <c r="E8" s="30" t="inlineStr">
+        <is>
+          <t>https://jainmetalgroup.com/trading.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1" s="15">
+      <c r="A9" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>MTC Group</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>India (location not confirmed)</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="inlineStr">
+        <is>
+          <t>Non-ferrous scrap: aluminium, zinc, brass, copper</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>https://www.mtcgroup.in/non-ferrous-scrap.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1" s="15">
+      <c r="A10" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>Kamala Trading Co</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>Howrah, West Bengal</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="inlineStr">
+        <is>
+          <t>Gunmetal/bronze scrap, copper cable and wire scrap, brass scrap</t>
+        </is>
+      </c>
+      <c r="E10" s="30" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/kamalatradingco</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1" s="15">
+      <c r="A11" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>Raameshth Enterprise</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>Howrah, West Bengal</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="inlineStr">
+        <is>
+          <t>Gunmetal, bronze, aluminium bronze and copper-nickel scrap</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/raameshthenterprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1" s="15">
+      <c r="A12" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>Metal Scrap India</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>Jamnagar, Gujarat</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
+          <t>Brass, copper and brass mix, gunmetal, aluminium bronze scrap (including UK-import gunmetal)</t>
+        </is>
+      </c>
+      <c r="E12" s="30" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/metalscrapindia</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1" s="15">
+      <c r="A13" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>P R International</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="inlineStr">
+        <is>
+          <t>Dared, Jamnagar, Gujarat</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>Brass scrap, gunmetal scrap, bronze scrap, copper alloy ingot</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/printernational</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1" s="15">
+      <c r="A14" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>Sona Metals</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>Brass, copper and aluminium products; brass scrap sales (trading since 1999)</t>
+        </is>
+      </c>
+      <c r="E14" s="30" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/sonametals/testimonial.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1" s="15">
+      <c r="A15" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>Jaimin Enterprise CSC (JE Metal Trade)</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="inlineStr">
+        <is>
+          <t>Bhuj, Gujarat</t>
+        </is>
+      </c>
+      <c r="D15" s="25" t="inlineStr">
+        <is>
+          <t>Copper millberry wire scrap and aluminium extrusion 6063 scrap</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>https://www.globallinker.com/seller/jaimin-enterprise-csc</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1" s="15">
+      <c r="A16" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>Shreeji Sales</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>Ferrous and non-ferrous scrap; wants copper millberry volumes (port: Mundra)</t>
+        </is>
+      </c>
+      <c r="E16" s="30" t="inlineStr">
+        <is>
+          <t>https://www.recycleinme.com/rim-namanmetal/home</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1" s="15">
+      <c r="A17" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>DCExporter</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="D17" s="25" t="inlineStr">
+        <is>
+          <t>Copper millberry wire scrap, copper cathode, aluminium ingot</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>https://www.globallinker.com/products/copper-mulberry-wire-scrap-8544193</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1" s="15">
+      <c r="A18" s="27" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>Pragna Overseas Ventures</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>Kolkata, West Bengal</t>
+        </is>
+      </c>
+      <c r="D18" s="29" t="inlineStr">
+        <is>
+          <t>Aluminium extrusion, wheel, UBC and radiator scrap</t>
+        </is>
+      </c>
+      <c r="E18" s="30" t="inlineStr">
+        <is>
+          <t>https://www.alcircle.com/biz/profile/pragna-overseas-ventures-18442</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1" s="15">
+      <c r="A19" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>Lucky Aluminium</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D19" s="25" t="inlineStr">
+        <is>
+          <t>Aluminium extrusion 6063, UBC and turning scrap</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>https://www.alcircle.com/biz/biz/profile/lucky-aluminium-39214</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1" s="15">
+      <c r="A20" s="27" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>MET India</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="inlineStr">
+        <is>
+          <t>Aluminium extrusion 6063, tense, taint-tabor and foil scrap</t>
+        </is>
+      </c>
+      <c r="E20" s="30" t="inlineStr">
+        <is>
+          <t>https://www.alcircle.com/biz/profile/met-india-34770</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1" s="15">
+      <c r="A21" s="23" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>Metal Paradise</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="inlineStr">
+        <is>
+          <t>Prince Road, Moradabad, Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="D21" s="25" t="inlineStr">
+        <is>
+          <t>Brass scrap (listed at Rs 520/kg, price not verified)</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>https://www.dial4trade.com/uttar-pradesh/scrap-dealers.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1" s="15">
+      <c r="A22" s="27" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="28" t="inlineStr">
+        <is>
+          <t>Welspring Universal</t>
+        </is>
+      </c>
+      <c r="C22" s="29" t="inlineStr">
+        <is>
+          <t>Mayapuri, Delhi</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
+        <is>
+          <t>Brass scrap and brass products</t>
+        </is>
+      </c>
+      <c r="E22" s="30" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/delhi/brass-scrap.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1" s="15">
+      <c r="A23" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>Guru Krupa Metal</t>
+        </is>
+      </c>
+      <c r="C23" s="25" t="inlineStr">
+        <is>
+          <t>Khyala, Delhi</t>
+        </is>
+      </c>
+      <c r="D23" s="25" t="inlineStr">
+        <is>
+          <t>Brass scrap</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/delhi/brass-scrap.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1" s="15">
+      <c r="A24" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="28" t="inlineStr">
+        <is>
+          <t>S.J Metal</t>
+        </is>
+      </c>
+      <c r="C24" s="29" t="inlineStr">
+        <is>
+          <t>Bali Nagar, Delhi</t>
+        </is>
+      </c>
+      <c r="D24" s="29" t="inlineStr">
+        <is>
+          <t>Brass scrap</t>
+        </is>
+      </c>
+      <c r="E24" s="30" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/delhi/brass-scrap.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1" s="15">
+      <c r="A25" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Shiv Metal Foundry</t>
+        </is>
+      </c>
+      <c r="C25" s="25" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="D25" s="25" t="inlineStr">
+        <is>
+          <t>Bronze scrap (listed at Rs 600/kg, price not verified)</t>
+        </is>
+      </c>
+      <c r="E25" s="26" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/impcat/bronze-scrap.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1" s="15">
+      <c r="A26" s="27" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="28" t="inlineStr">
+        <is>
+          <t>Mukesh Metal Corporation</t>
+        </is>
+      </c>
+      <c r="C26" s="29" t="inlineStr">
+        <is>
+          <t>Mumbai, Maharashtra</t>
+        </is>
+      </c>
+      <c r="D26" s="29" t="inlineStr">
+        <is>
+          <t>Phosphor bronze scrap pieces for melting (85% copper or more)</t>
+        </is>
+      </c>
+      <c r="E26" s="30" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/impcat/bronze-scrap.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="40" customHeight="1" s="15">
+      <c r="A27" s="23" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>Metcast India</t>
+        </is>
+      </c>
+      <c r="C27" s="25" t="inlineStr">
+        <is>
+          <t>Howrah, West Bengal</t>
+        </is>
+      </c>
+      <c r="D27" s="25" t="inlineStr">
+        <is>
+          <t>Bronze, brass and gunmetal scrap (listed at Rs 900/kg, 100 kg minimum; price not verified)</t>
+        </is>
+      </c>
+      <c r="E27" s="26" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/impcat/bronze-scrap.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="40" customHeight="1" s="15">
+      <c r="A28" s="27" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>Ronak Enterprise</t>
+        </is>
+      </c>
+      <c r="C28" s="29" t="inlineStr">
+        <is>
+          <t>Bhavnagar, Gujarat</t>
+        </is>
+      </c>
+      <c r="D28" s="29" t="inlineStr">
+        <is>
+          <t>Gunmetal bronze scrap (listed at Rs 900/kg in 50 kg packs; price not verified)</t>
+        </is>
+      </c>
+      <c r="E28" s="30" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/impcat/bronze-scrap.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="40" customHeight="1" s="15">
+      <c r="A29" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>Gaurav Steel</t>
+        </is>
+      </c>
+      <c r="C29" s="25" t="inlineStr">
+        <is>
+          <t>Kolkata, West Bengal</t>
+        </is>
+      </c>
+      <c r="D29" s="25" t="inlineStr">
+        <is>
+          <t>Phosphor bronze scrap (listed at Rs 750/kg in 50 kg bags; price not verified)</t>
+        </is>
+      </c>
+      <c r="E29" s="26" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/impcat/bronze-scrap.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="40" customHeight="1" s="15">
+      <c r="A30" s="27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="28" t="inlineStr">
+        <is>
+          <t>Prashaant Steel &amp; Alloys</t>
+        </is>
+      </c>
+      <c r="C30" s="29" t="inlineStr">
+        <is>
+          <t>Madhavbaug, Mumbai</t>
+        </is>
+      </c>
+      <c r="D30" s="29" t="inlineStr">
+        <is>
+          <t>Phosphor bronze blocks and ingots (listed at Rs 600/kg); ingot, not scrap</t>
+        </is>
+      </c>
+      <c r="E30" s="30" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/impcat/bronze-ingots.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="40" customHeight="1" s="15">
+      <c r="A31" s="23" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>Supreme Metals</t>
+        </is>
+      </c>
+      <c r="C31" s="25" t="inlineStr">
+        <is>
+          <t>India (location not confirmed)</t>
+        </is>
+      </c>
+      <c r="D31" s="25" t="inlineStr">
+        <is>
+          <t>Metal trader appearing in brass and bronze scrap searches</t>
+        </is>
+      </c>
+      <c r="E31" s="26" t="inlineStr">
+        <is>
+          <t>https://m.indiamart.com/supreme-metals/testimonial.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="40" customHeight="1" s="15">
+      <c r="A32" s="27" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>Laxmi Alloys Casting Co</t>
+        </is>
+      </c>
+      <c r="C32" s="29" t="inlineStr">
+        <is>
+          <t>India (location not confirmed)</t>
+        </is>
+      </c>
+      <c r="D32" s="29" t="inlineStr">
+        <is>
+          <t>Alloy casting company appearing in gunmetal and bronze searches</t>
+        </is>
+      </c>
+      <c r="E32" s="30" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/laxmi-alloys-casting-co-9667818/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="40" customHeight="1" s="15">
+      <c r="A33" s="23" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>Kqer Manglam Metals</t>
+        </is>
+      </c>
+      <c r="C33" s="25" t="inlineStr">
+        <is>
+          <t>India (location not confirmed)</t>
+        </is>
+      </c>
+      <c r="D33" s="25" t="inlineStr">
+        <is>
+          <t>Copper alloy supplier appearing in bronze scrap searches</t>
+        </is>
+      </c>
+      <c r="E33" s="26" t="inlineStr">
+        <is>
+          <t>https://matmatch.com/suppliers/kqer-manglam-metals</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="40" customHeight="1" s="15">
+      <c r="A34" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>Enlighten Businesses Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="inlineStr">
+        <is>
+          <t>Dared, Jamnagar, Gujarat</t>
+        </is>
+      </c>
+      <c r="D34" s="29" t="inlineStr">
+        <is>
+          <t>Gunmetal scrap</t>
+        </is>
+      </c>
+      <c r="E34" s="30" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/indian-suppliers/gunmetal-scrap.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="40" customHeight="1" s="15">
+      <c r="A35" s="23" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>Kernel Serviced</t>
+        </is>
+      </c>
+      <c r="C35" s="25" t="inlineStr">
+        <is>
+          <t>Noida, Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="D35" s="25" t="inlineStr">
+        <is>
+          <t>Gunmetal scrap for foundry use (no price shown)</t>
+        </is>
+      </c>
+      <c r="E35" s="26" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/indian-suppliers/gunmetal-scrap.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="40" customHeight="1" s="15">
+      <c r="A36" s="27" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="28" t="inlineStr">
+        <is>
+          <t>Rajesh Metal Syndicate</t>
+        </is>
+      </c>
+      <c r="C36" s="29" t="inlineStr">
+        <is>
+          <t>Mumbai, Maharashtra</t>
+        </is>
+      </c>
+      <c r="D36" s="29" t="inlineStr">
+        <is>
+          <t>Commercial gunmetal scrap (listed at Rs 41/kg, 100 kg minimum; price looks unusually low, verify)</t>
+        </is>
+      </c>
+      <c r="E36" s="30" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/indian-suppliers/gunmetal-scrap.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="40" customHeight="1" s="15">
+      <c r="A37" s="23" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="24" t="inlineStr">
+        <is>
+          <t>Shanky Group</t>
+        </is>
+      </c>
+      <c r="C37" s="25" t="inlineStr">
+        <is>
+          <t>Ashok Vihar, Delhi</t>
+        </is>
+      </c>
+      <c r="D37" s="25" t="inlineStr">
+        <is>
+          <t>Brass scrap</t>
+        </is>
+      </c>
+      <c r="E37" s="26" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/delhi/brass-scrap.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="40" customHeight="1" s="15">
+      <c r="A38" s="27" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="28" t="inlineStr">
+        <is>
+          <t>Vansi Iron Traders</t>
+        </is>
+      </c>
+      <c r="C38" s="29" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D38" s="29" t="inlineStr">
+        <is>
+          <t>Scrap trader appearing in the Delhi brass scrap listing</t>
+        </is>
+      </c>
+      <c r="E38" s="30" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/delhi/brass-scrap.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="40" customHeight="1" s="15">
+      <c r="A39" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>Prism Metals</t>
+        </is>
+      </c>
+      <c r="C39" s="25" t="inlineStr">
+        <is>
+          <t>B-28 Mayapuri Industrial Area, Phase-1, New Delhi</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="inlineStr">
+        <is>
+          <t>Brass products manufacturer (not a scrap dealer)</t>
+        </is>
+      </c>
+      <c r="E39" s="26" t="inlineStr">
+        <is>
+          <t>https://www.exportersindia.com/delhi/brass-scrap.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="40" customHeight="1" s="15">
+      <c r="A40" s="27" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="28" t="inlineStr">
+        <is>
+          <t>S.D. Industrial Corporation</t>
+        </is>
+      </c>
+      <c r="C40" s="29" t="inlineStr">
+        <is>
+          <t>India (location not confirmed)</t>
+        </is>
+      </c>
+      <c r="D40" s="29" t="inlineStr">
+        <is>
+          <t>Aluminium alloy wheel, 6063, wire and UBC scrap</t>
+        </is>
+      </c>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>https://www.alcircle.com/biz/verified-aluminium-suppliers?pageNo=8</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="40" customHeight="1" s="15">
+      <c r="A41" s="23" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="24" t="inlineStr">
+        <is>
+          <t>Elevare Exports and Imports</t>
+        </is>
+      </c>
+      <c r="C41" s="25" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="D41" s="25" t="inlineStr">
+        <is>
+          <t>Aluminium extrusion scrap 6063/6061 (1 MT minimum)</t>
+        </is>
+      </c>
+      <c r="E41" s="26" t="inlineStr">
+        <is>
+          <t>https://www.globallinker.com/seller/elevare-exports-and-imports</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="40" customHeight="1" s="15">
+      <c r="A42" s="27" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="28" t="inlineStr">
+        <is>
+          <t>Century Metal Recycling Ltd</t>
+        </is>
+      </c>
+      <c r="C42" s="29" t="inlineStr">
+        <is>
+          <t>Faridabad, Haryana</t>
+        </is>
+      </c>
+      <c r="D42" s="29" t="inlineStr">
+        <is>
+          <t>Aluminium and zinc alloy recycler; sells ingot or molten metal (no copper or brass)</t>
+        </is>
+      </c>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>https://www.instafinancials.com/company/century-metal-recycling-limited/U74899HR1994PLC086105</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:E42"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId38"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>

</xml_diff>

<commit_message>
Add Auction Sites by Alloy sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XVi8LRrXHdPJmY1JXLxuUU
</commit_message>
<xml_diff>
--- a/Private_Scrap_Auction_Links_updated.xlsx
+++ b/Private_Scrap_Auction_Links_updated.xlsx
@@ -10,13 +10,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Less Relevant" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scrap Vendors" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendor List" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auction Sites by Alloy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Highly Relevant'!$A$4:$L$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Less Relevant'!$A$4:$L$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scrap Vendors'!$A$4:$G$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Vendor List'!$A$4:$E$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auction Sites by Alloy'!$A$10:$I$39</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -27,7 +29,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,8 +86,19 @@
       <sz val="10"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B0522A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00B0522A"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -135,8 +148,13 @@
         <fgColor rgb="00F2F6FA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -182,11 +200,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -265,6 +327,24 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7593,6 +7673,1331 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00B0522A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" style="15" min="1" max="1"/>
+    <col width="30" customWidth="1" style="15" min="2" max="2"/>
+    <col width="46" customWidth="1" style="15" min="3" max="3"/>
+    <col width="26" customWidth="1" style="15" min="4" max="4"/>
+    <col width="14" customWidth="1" style="15" min="5" max="5"/>
+    <col width="16" customWidth="1" style="15" min="6" max="6"/>
+    <col width="12" customWidth="1" style="15" min="7" max="7"/>
+    <col width="14" customWidth="1" style="15" min="8" max="8"/>
+    <col width="60" customWidth="1" style="15" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Auction sites for the C97600 and C99700 alloy inputs</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="n"/>
+      <c r="C1" s="20" t="n"/>
+      <c r="D1" s="20" t="n"/>
+      <c r="E1" s="20" t="n"/>
+      <c r="F1" s="20" t="n"/>
+      <c r="G1" s="20" t="n"/>
+      <c r="H1" s="20" t="n"/>
+      <c r="I1" s="20" t="n"/>
+    </row>
+    <row r="2" ht="50" customHeight="1" s="15">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>You did not list the alloys, so this sheet assumes C97600 and C99700 and the scrap that feeds them. Marks: ● = this scrap type was seen in lots on the site (from the Highly Relevant and Less Relevant sheets); ○ = possible, not seen; blank = not expected. Sites marked New were found on 23 Oct 2026 by web search and not yet checked for live lots. Most private sites show lot details only after registration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>What each alloy needs from scrap</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>Alloy</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>Composition (main elements)</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>Scrap to look for</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="n"/>
+      <c r="E5" s="32" t="n"/>
+      <c r="F5" s="32" t="n"/>
+      <c r="G5" s="32" t="n"/>
+      <c r="H5" s="32" t="n"/>
+      <c r="I5" s="33" t="n"/>
+    </row>
+    <row r="6" ht="32" customHeight="1" s="15">
+      <c r="A6" s="34" t="inlineStr">
+        <is>
+          <t>C97600</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>Cu 63-67, Ni 19-21.5, Zn 3-9, Sn 3.5-4.5, Pb 3-5</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>Copper scrap and cable; nickel or cupro-nickel and nickel-silver scrap; bronze or gunmetal (tin); brass (zinc); leaded scrap</t>
+        </is>
+      </c>
+      <c r="D6" s="32" t="n"/>
+      <c r="E6" s="32" t="n"/>
+      <c r="F6" s="32" t="n"/>
+      <c r="G6" s="32" t="n"/>
+      <c r="H6" s="32" t="n"/>
+      <c r="I6" s="33" t="n"/>
+    </row>
+    <row r="7" ht="32" customHeight="1" s="15">
+      <c r="A7" s="34" t="inlineStr">
+        <is>
+          <t>C99700</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Cu 54-60, Zn 19-25, Mn 11-15, Ni 4-6, Al 0.5-3</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>Copper and brass scrap; zinc; aluminium scrap (small share); nickel scrap. Manganese has no scrap source, so buy it as master alloy</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="n"/>
+      <c r="E7" s="32" t="n"/>
+      <c r="F7" s="32" t="n"/>
+      <c r="G7" s="32" t="n"/>
+      <c r="H7" s="32" t="n"/>
+      <c r="I7" s="33" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="31" t="inlineStr">
+        <is>
+          <t>Auction sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>Auction site</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>Copper (cable, windings)</t>
+        </is>
+      </c>
+      <c r="F10" s="22" t="inlineStr">
+        <is>
+          <t>Brass / bronze / gunmetal</t>
+        </is>
+      </c>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>Aluminium</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="inlineStr">
+        <is>
+          <t>Nickel / cupro-nickel</t>
+        </is>
+      </c>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1" s="15">
+      <c r="A11" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="36" t="inlineStr">
+        <is>
+          <t>MSTC e-commerce</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>https://www.mstcindia.co.in/content/ecommerce_services.aspx</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="inlineStr">
+        <is>
+          <t>Government / PSU forward e-auctions</t>
+        </is>
+      </c>
+      <c r="E11" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G11" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H11" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="I11" s="25" t="inlineStr">
+        <is>
+          <t>Main channel for central and state PSU non-ferrous scrap; buyer registration with GSTIN and PAN [New]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1" s="15">
+      <c r="A12" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="36" t="inlineStr">
+        <is>
+          <t>mjunction</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>https://www.mjunction.in/</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
+          <t>Industrial e-auction service</t>
+        </is>
+      </c>
+      <c r="E12" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F12" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G12" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H12" s="38" t="inlineStr"/>
+      <c r="I12" s="29" t="inlineStr">
+        <is>
+          <t>Runs e-auctions for ferrous and non-ferrous scrap for large corporates; says over 6,000 registered buyers [New]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1" s="15">
+      <c r="A13" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="36" t="inlineStr">
+        <is>
+          <t>Recykal metal marketplace</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>https://www.recykal.com/marketplace-metal-buyer</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>Buyer-side marketplace</t>
+        </is>
+      </c>
+      <c r="E13" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F13" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G13" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H13" s="37" t="inlineStr"/>
+      <c r="I13" s="25" t="inlineStr">
+        <is>
+          <t>Lists copper, aluminium, lead, brass and zinc from GST-compliant sellers [New]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44" customHeight="1" s="15">
+      <c r="A14" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>Right2Vote e-Auction</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>https://right2vote.in/scrap-eauction-platform-for-transparent-online-scrap-auctions/</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>Auction software for sellers</t>
+        </is>
+      </c>
+      <c r="E14" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F14" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G14" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H14" s="38" t="inlineStr"/>
+      <c r="I14" s="29" t="inlineStr">
+        <is>
+          <t>Platform plants use to run their own scrap auctions; approved bidders only [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1" s="15">
+      <c r="A15" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>Matex Technologies</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>https://matextechnologies.com/e-auctions/</t>
+        </is>
+      </c>
+      <c r="D15" s="25" t="inlineStr">
+        <is>
+          <t>Private e-auctions</t>
+        </is>
+      </c>
+      <c r="E15" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F15" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G15" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H15" s="37" t="inlineStr"/>
+      <c r="I15" s="25" t="inlineStr">
+        <is>
+          <t>Copper windings, brass, aluminium, wire harness lots across India [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="44" customHeight="1" s="15">
+      <c r="A16" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>Salasar Auction</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>https://salasarauction.com/forward-auction-list</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>Private e-auctions</t>
+        </is>
+      </c>
+      <c r="E16" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F16" s="38" t="inlineStr"/>
+      <c r="G16" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H16" s="38" t="inlineStr"/>
+      <c r="I16" s="29" t="inlineStr">
+        <is>
+          <t>Copper scrap, XLPE and wire cable, motors; lots visible after login [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="44" customHeight="1" s="15">
+      <c r="A17" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>Neelami Auctioneer</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>https://www.neelami.co.in</t>
+        </is>
+      </c>
+      <c r="D17" s="25" t="inlineStr">
+        <is>
+          <t>Corporate scrap auctions</t>
+        </is>
+      </c>
+      <c r="E17" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F17" s="37" t="inlineStr"/>
+      <c r="G17" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H17" s="37" t="inlineStr"/>
+      <c r="I17" s="25" t="inlineStr">
+        <is>
+          <t>Copper cable and scrap for Grasim, L&amp;T, Adani; lot lists are PDFs [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="44" customHeight="1" s="15">
+      <c r="A18" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>Select eAuctioneer</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>https://www.eauctioneer.in</t>
+        </is>
+      </c>
+      <c r="D18" s="29" t="inlineStr">
+        <is>
+          <t>Private e-auctions</t>
+        </is>
+      </c>
+      <c r="E18" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F18" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G18" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H18" s="38" t="inlineStr"/>
+      <c r="I18" s="29" t="inlineStr">
+        <is>
+          <t>Elin Electronics lots: aluminium, motors, AC coils [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="44" customHeight="1" s="15">
+      <c r="A19" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>INTIS Online Auctions</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>https://www.intis.in/</t>
+        </is>
+      </c>
+      <c r="D19" s="25" t="inlineStr">
+        <is>
+          <t>Private e-auctions</t>
+        </is>
+      </c>
+      <c r="E19" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F19" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G19" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H19" s="37" t="inlineStr"/>
+      <c r="I19" s="25" t="inlineStr">
+        <is>
+          <t>Brass scrap and wire, several copper grades, aluminium; Karnataka lots [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1" s="15">
+      <c r="A20" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>Steelez</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>https://user.steelez.com/bidder/auction-detail</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="inlineStr">
+        <is>
+          <t>Private e-auctions</t>
+        </is>
+      </c>
+      <c r="E20" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F20" s="38" t="inlineStr"/>
+      <c r="G20" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H20" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I20" s="29" t="inlineStr">
+        <is>
+          <t>Copper in electrical scrap, aluminium, and a nickel / e-waste lot [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44" customHeight="1" s="15">
+      <c r="A21" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>SalvorSettlers</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>https://salvorsettlers.com</t>
+        </is>
+      </c>
+      <c r="D21" s="25" t="inlineStr">
+        <is>
+          <t>Insurance salvage</t>
+        </is>
+      </c>
+      <c r="E21" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F21" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G21" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H21" s="37" t="inlineStr"/>
+      <c r="I21" s="25" t="inlineStr">
+        <is>
+          <t>AC coils (copper and brass), transformer windings, fire-affected copper and aluminium [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1" s="15">
+      <c r="A22" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="B22" s="28" t="inlineStr">
+        <is>
+          <t>Sealthedeal</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>https://www.sealthedeal.co.in</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
+        <is>
+          <t>Insurance salvage</t>
+        </is>
+      </c>
+      <c r="E22" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F22" s="38" t="inlineStr"/>
+      <c r="G22" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H22" s="38" t="inlineStr"/>
+      <c r="I22" s="29" t="inlineStr">
+        <is>
+          <t>Fire-affected cable and stabilizer windings, priced per kg [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="44" customHeight="1" s="15">
+      <c r="A23" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>The Salvage Bids</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>https://thesalvagebids.com</t>
+        </is>
+      </c>
+      <c r="D23" s="25" t="inlineStr">
+        <is>
+          <t>Insurance salvage</t>
+        </is>
+      </c>
+      <c r="E23" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F23" s="37" t="inlineStr"/>
+      <c r="G23" s="37" t="inlineStr"/>
+      <c r="H23" s="37" t="inlineStr"/>
+      <c r="I23" s="25" t="inlineStr">
+        <is>
+          <t>Damaged transformers and plant; bid per lot or per MT [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="44" customHeight="1" s="15">
+      <c r="A24" s="27" t="n">
+        <v>14</v>
+      </c>
+      <c r="B24" s="28" t="inlineStr">
+        <is>
+          <t>Indian Salvage Settlers</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr">
+        <is>
+          <t>https://indiansalvagesettler.com/Auction.aspx</t>
+        </is>
+      </c>
+      <c r="D24" s="29" t="inlineStr">
+        <is>
+          <t>Insurance salvage</t>
+        </is>
+      </c>
+      <c r="E24" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F24" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G24" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H24" s="38" t="inlineStr"/>
+      <c r="I24" s="29" t="inlineStr">
+        <is>
+          <t>Copper wire, aluminium, AC coils (past lots shown) [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="44" customHeight="1" s="15">
+      <c r="A25" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Canrod Metals</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>https://auction.canrod.com/</t>
+        </is>
+      </c>
+      <c r="D25" s="25" t="inlineStr">
+        <is>
+          <t>Private e-auctions</t>
+        </is>
+      </c>
+      <c r="E25" s="37" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F25" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G25" s="37" t="inlineStr"/>
+      <c r="H25" s="37" t="inlineStr"/>
+      <c r="I25" s="25" t="inlineStr">
+        <is>
+          <t>Motors and e-waste with copper; seller names masked [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="44" customHeight="1" s="15">
+      <c r="A26" s="27" t="n">
+        <v>16</v>
+      </c>
+      <c r="B26" s="28" t="inlineStr">
+        <is>
+          <t>MSP Auction</t>
+        </is>
+      </c>
+      <c r="C26" s="30" t="inlineStr">
+        <is>
+          <t>https://mspauction.com/auctions</t>
+        </is>
+      </c>
+      <c r="D26" s="29" t="inlineStr">
+        <is>
+          <t>Private e-auctions</t>
+        </is>
+      </c>
+      <c r="E26" s="38" t="inlineStr"/>
+      <c r="F26" s="38" t="inlineStr"/>
+      <c r="G26" s="38" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H26" s="38" t="inlineStr"/>
+      <c r="I26" s="29" t="inlineStr">
+        <is>
+          <t>Aluminium and aluminium cable lots from Quality Alloys (closed) [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="44" customHeight="1" s="15">
+      <c r="A27" s="23" t="n">
+        <v>17</v>
+      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>CarTrade Exchange</t>
+        </is>
+      </c>
+      <c r="C27" s="26" t="inlineStr">
+        <is>
+          <t>https://www.cartradeexchange.com/</t>
+        </is>
+      </c>
+      <c r="D27" s="25" t="inlineStr">
+        <is>
+          <t>Vehicle salvage</t>
+        </is>
+      </c>
+      <c r="E27" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F27" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G27" s="37" t="inlineStr"/>
+      <c r="H27" s="37" t="inlineStr"/>
+      <c r="I27" s="25" t="inlineStr">
+        <is>
+          <t>Copper and brass in radiators and wiring; low relevance [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="44" customHeight="1" s="15">
+      <c r="A28" s="27" t="n">
+        <v>18</v>
+      </c>
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>eAuctionsIndia</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr">
+        <is>
+          <t>https://www.eauctionsindia.com</t>
+        </is>
+      </c>
+      <c r="D28" s="29" t="inlineStr">
+        <is>
+          <t>Bank / SARFAESI listings</t>
+        </is>
+      </c>
+      <c r="E28" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F28" s="38" t="inlineStr"/>
+      <c r="G28" s="38" t="inlineStr"/>
+      <c r="H28" s="38" t="inlineStr"/>
+      <c r="I28" s="29" t="inlineStr">
+        <is>
+          <t>Plant and electrical units; copper not itemised [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="44" customHeight="1" s="15">
+      <c r="A29" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>BidMyScrap</t>
+        </is>
+      </c>
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>https://bidmyscrap.com/home/upcomingAuction</t>
+        </is>
+      </c>
+      <c r="D29" s="25" t="inlineStr">
+        <is>
+          <t>Private e-auctions</t>
+        </is>
+      </c>
+      <c r="E29" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F29" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G29" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H29" s="37" t="inlineStr"/>
+      <c r="I29" s="25" t="inlineStr">
+        <is>
+          <t>Lots visible only after registration [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="44" customHeight="1" s="15">
+      <c r="A30" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="B30" s="28" t="inlineStr">
+        <is>
+          <t>Auction-it (JindalX)</t>
+        </is>
+      </c>
+      <c r="C30" s="30" t="inlineStr">
+        <is>
+          <t>https://www.auctionit.ai/auctions</t>
+        </is>
+      </c>
+      <c r="D30" s="29" t="inlineStr">
+        <is>
+          <t>Private e-auctions</t>
+        </is>
+      </c>
+      <c r="E30" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F30" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G30" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H30" s="38" t="inlineStr"/>
+      <c r="I30" s="29" t="inlineStr">
+        <is>
+          <t>Auction list showed a server error on 11 Oct [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="44" customHeight="1" s="15">
+      <c r="A31" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>ScrapDekho</t>
+        </is>
+      </c>
+      <c r="C31" s="26" t="inlineStr">
+        <is>
+          <t>https://scrapdekho.com/</t>
+        </is>
+      </c>
+      <c r="D31" s="25" t="inlineStr">
+        <is>
+          <t>Private e-auctions</t>
+        </is>
+      </c>
+      <c r="E31" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F31" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G31" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H31" s="37" t="inlineStr"/>
+      <c r="I31" s="25" t="inlineStr">
+        <is>
+          <t>Lots shown after login [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="44" customHeight="1" s="15">
+      <c r="A32" s="27" t="n">
+        <v>22</v>
+      </c>
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>Auction India (TVS Electronics)</t>
+        </is>
+      </c>
+      <c r="C32" s="30" t="inlineStr">
+        <is>
+          <t>https://www.auctionindia.com/</t>
+        </is>
+      </c>
+      <c r="D32" s="29" t="inlineStr">
+        <is>
+          <t>Private e-auctions</t>
+        </is>
+      </c>
+      <c r="E32" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F32" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G32" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H32" s="38" t="inlineStr"/>
+      <c r="I32" s="29" t="inlineStr">
+        <is>
+          <t>Metal and e-waste lots; also used by some government bodies [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="44" customHeight="1" s="15">
+      <c r="A33" s="23" t="n">
+        <v>23</v>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>Spotbid</t>
+        </is>
+      </c>
+      <c r="C33" s="26" t="inlineStr">
+        <is>
+          <t>https://www.spotbid.in/Auction.aspx</t>
+        </is>
+      </c>
+      <c r="D33" s="25" t="inlineStr">
+        <is>
+          <t>Private e-auctions</t>
+        </is>
+      </c>
+      <c r="E33" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F33" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G33" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H33" s="37" t="inlineStr"/>
+      <c r="I33" s="25" t="inlineStr">
+        <is>
+          <t>Scrapped assets; items not itemised [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="44" customHeight="1" s="15">
+      <c r="A34" s="27" t="n">
+        <v>24</v>
+      </c>
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>Auctions by Pahwa</t>
+        </is>
+      </c>
+      <c r="C34" s="30" t="inlineStr">
+        <is>
+          <t>https://www.auctionsbypahwa.com/</t>
+        </is>
+      </c>
+      <c r="D34" s="29" t="inlineStr">
+        <is>
+          <t>On-site and online auctions</t>
+        </is>
+      </c>
+      <c r="E34" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F34" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G34" s="38" t="inlineStr"/>
+      <c r="H34" s="38" t="inlineStr"/>
+      <c r="I34" s="29" t="inlineStr">
+        <is>
+          <t>Industrial scrap and machinery in Delhi NCR [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="44" customHeight="1" s="15">
+      <c r="A35" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>Just Auction</t>
+        </is>
+      </c>
+      <c r="C35" s="26" t="inlineStr">
+        <is>
+          <t>https://www.justauction.in/</t>
+        </is>
+      </c>
+      <c r="D35" s="25" t="inlineStr">
+        <is>
+          <t>Private auctions and tenders</t>
+        </is>
+      </c>
+      <c r="E35" s="37" t="inlineStr"/>
+      <c r="F35" s="37" t="inlineStr"/>
+      <c r="G35" s="37" t="inlineStr"/>
+      <c r="H35" s="37" t="inlineStr"/>
+      <c r="I35" s="25" t="inlineStr">
+        <is>
+          <t>No relevant material on 11 Oct; check later [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="44" customHeight="1" s="15">
+      <c r="A36" s="27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B36" s="28" t="inlineStr">
+        <is>
+          <t>SalvageHub</t>
+        </is>
+      </c>
+      <c r="C36" s="30" t="inlineStr">
+        <is>
+          <t>https://salvagehub.in/</t>
+        </is>
+      </c>
+      <c r="D36" s="29" t="inlineStr">
+        <is>
+          <t>Insurance salvage</t>
+        </is>
+      </c>
+      <c r="E36" s="38" t="inlineStr"/>
+      <c r="F36" s="38" t="inlineStr"/>
+      <c r="G36" s="38" t="inlineStr"/>
+      <c r="H36" s="38" t="inlineStr"/>
+      <c r="I36" s="29" t="inlineStr">
+        <is>
+          <t>Industrial assets; no readable lots on 11 Oct [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="44" customHeight="1" s="15">
+      <c r="A37" s="23" t="n">
+        <v>27</v>
+      </c>
+      <c r="B37" s="24" t="inlineStr">
+        <is>
+          <t>Maxsure Bidders</t>
+        </is>
+      </c>
+      <c r="C37" s="26" t="inlineStr">
+        <is>
+          <t>https://maxsurebidders.com/bid/wire-coils</t>
+        </is>
+      </c>
+      <c r="D37" s="25" t="inlineStr">
+        <is>
+          <t>Insurance salvage</t>
+        </is>
+      </c>
+      <c r="E37" s="37" t="inlineStr"/>
+      <c r="F37" s="37" t="inlineStr"/>
+      <c r="G37" s="37" t="inlineStr"/>
+      <c r="H37" s="37" t="inlineStr"/>
+      <c r="I37" s="25" t="inlineStr">
+        <is>
+          <t>Wire coils, probably steel; low relevance [In workbook]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="44" customHeight="1" s="15">
+      <c r="A38" s="27" t="n">
+        <v>28</v>
+      </c>
+      <c r="B38" s="36" t="inlineStr">
+        <is>
+          <t>ScrapBays (UK)</t>
+        </is>
+      </c>
+      <c r="C38" s="30" t="inlineStr">
+        <is>
+          <t>https://www.letsrecycle.com/supplier/scrapbays-ltd/</t>
+        </is>
+      </c>
+      <c r="D38" s="29" t="inlineStr">
+        <is>
+          <t>International scrap auctions</t>
+        </is>
+      </c>
+      <c r="E38" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F38" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G38" s="38" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H38" s="38" t="inlineStr"/>
+      <c r="I38" s="29" t="inlineStr">
+        <is>
+          <t>London-based bulk-lot auction platform; listed as launch-stage; directory page shown because its own site was not found [New]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="44" customHeight="1" s="15">
+      <c r="A39" s="23" t="n">
+        <v>29</v>
+      </c>
+      <c r="B39" s="36" t="inlineStr">
+        <is>
+          <t>MetalsPlace (international)</t>
+        </is>
+      </c>
+      <c r="C39" s="26" t="inlineStr">
+        <is>
+          <t>https://metalsplace.com/listings/brass-scrap/united-kingdom</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="inlineStr">
+        <is>
+          <t>International B2B listings</t>
+        </is>
+      </c>
+      <c r="E39" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F39" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G39" s="37" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H39" s="37" t="inlineStr"/>
+      <c r="I39" s="25" t="inlineStr">
+        <is>
+          <t>Brass scrap listings from many countries; not an auction, use for sourcing leads [New]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A10:I39"/>
+  <mergeCells count="4">
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId29"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>

</xml_diff>